<commit_message>
I just opened and closed the .xlsx file, but it asked me if I wanted to save my changes.
</commit_message>
<xml_diff>
--- a/Inputs/CF_template_parameters_Exposure.xlsx
+++ b/Inputs/CF_template_parameters_Exposure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/bernstein_amanda_epa_gov/Documents/Documents/PKWG_models/pbpk_template_project/Inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="8_{21F6BD86-87FF-448A-B487-2BEC2C0D01E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C61C3420-DD52-4195-A1F1-B36A9D6295AC}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="8_{21F6BD86-87FF-448A-B487-2BEC2C0D01E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5482D379-EBDA-4B8D-9105-493C4F110ED8}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="28935" windowHeight="10785" activeTab="4" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Take_oral" sheetId="9" r:id="rId1"/>
@@ -408,16 +408,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
@@ -438,9 +429,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -478,7 +469,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -584,7 +575,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -726,7 +717,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -735,21 +726,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D6AAA3-4823-45FD-8570-D25DAB8AD8C8}">
   <dimension ref="A1:F39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.6328125" customWidth="1"/>
-    <col min="3" max="3" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -769,43 +760,43 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B2" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" t="s">
         <v>79</v>
       </c>
       <c r="F2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B3" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B4" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -815,14 +806,14 @@
       <c r="C5" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" t="s">
         <v>82</v>
       </c>
       <c r="F5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
@@ -832,14 +823,14 @@
       <c r="C6" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" t="s">
         <v>83</v>
       </c>
       <c r="F6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
@@ -849,28 +840,28 @@
       <c r="C7" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" t="s">
         <v>89</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" t="s">
         <v>71</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" t="s">
         <v>86</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>78</v>
       </c>
@@ -880,11 +871,11 @@
       <c r="C9" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>60</v>
       </c>
@@ -894,12 +885,11 @@
       <c r="C10" t="s">
         <v>61</v>
       </c>
-      <c r="E10" s="2"/>
       <c r="F10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>69</v>
       </c>
@@ -909,11 +899,11 @@
       <c r="C11" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>72</v>
       </c>
@@ -923,11 +913,11 @@
       <c r="C12" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>74</v>
       </c>
@@ -937,11 +927,11 @@
       <c r="C13" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -958,7 +948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -968,79 +958,79 @@
       <c r="C16" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16">
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="17" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" t="s">
         <v>93</v>
       </c>
-      <c r="D17" s="9">
-        <v>0</v>
-      </c>
-      <c r="E17" s="9">
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
         <v>0.27</v>
       </c>
     </row>
-    <row r="18" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18">
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="19" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" t="s">
         <v>99</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19">
         <v>298</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" t="s">
         <v>103</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20">
         <v>24450</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20">
         <v>24450</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1053,11 +1043,11 @@
       <c r="D21">
         <v>0</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21">
         <v>55</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1070,9 +1060,8 @@
       <c r="D22">
         <v>0</v>
       </c>
-      <c r="E22" s="4"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
@@ -1082,9 +1071,8 @@
       <c r="C23" t="s">
         <v>24</v>
       </c>
-      <c r="E23" s="4"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
@@ -1098,7 +1086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1108,11 +1096,11 @@
       <c r="D25">
         <v>0</v>
       </c>
-      <c r="E25" s="6">
+      <c r="E25">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
@@ -1126,7 +1114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
@@ -1140,8 +1128,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B28" t="s">
@@ -1151,7 +1139,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>64</v>
       </c>
@@ -1162,7 +1150,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>65</v>
       </c>
@@ -1173,7 +1161,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>67</v>
       </c>
@@ -1181,7 +1169,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
@@ -1192,7 +1180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
@@ -1203,7 +1191,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
@@ -1211,29 +1199,29 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="10" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" t="s">
         <v>57</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="36" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
@@ -1244,7 +1232,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>0</v>
       </c>
@@ -1264,529 +1252,528 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A49CAE4-A6EB-4905-A519-13D6D7FF729C}">
   <dimension ref="A1:F39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.6328125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="15.7265625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" style="6" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" style="6"/>
+    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="7" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" t="s">
         <v>79</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" t="s">
         <v>82</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" t="s">
         <v>83</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="7" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" t="s">
         <v>89</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" t="s">
         <v>71</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" t="s">
         <v>86</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" t="s">
         <v>76</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="7" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" t="s">
         <v>77</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="7" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="7" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" t="s">
         <v>75</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B15" s="7" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="7" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="8">
+      <c r="E16">
         <v>0.34722222222222221</v>
       </c>
     </row>
-    <row r="17" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" t="s">
         <v>93</v>
       </c>
-      <c r="D17" s="9">
-        <v>0</v>
-      </c>
-      <c r="E17" s="9">
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
         <v>0.27</v>
       </c>
     </row>
-    <row r="18" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18">
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="19" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" t="s">
         <v>99</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19">
         <v>298</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" t="s">
         <v>103</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20">
         <v>24450</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20">
         <v>24450</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="7" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="6">
-        <v>0</v>
-      </c>
-      <c r="E21" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="7" t="s">
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="7" t="s">
+      <c r="D22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="7" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="6">
-        <v>0</v>
-      </c>
-      <c r="E24" s="9">
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="7" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="6">
-        <v>0</v>
-      </c>
-      <c r="E25" s="6">
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="7" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="7" t="s">
+      <c r="D26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" t="s">
         <v>17</v>
       </c>
-      <c r="D27" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="10" t="s">
+      <c r="D27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E28">
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="7" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" t="s">
         <v>23</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="7" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="7" t="s">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="7" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" t="s">
         <v>47</v>
       </c>
-      <c r="D32" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="7" t="s">
+      <c r="D32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="7" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="10" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" t="s">
         <v>57</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="36" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="7" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" t="s">
         <v>59</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B39" s="7" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C39" s="7"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="7"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1796,529 +1783,528 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5A5AE8A-9C1B-4F50-8169-BE7AE9DBF28E}">
   <dimension ref="A1:F39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.6328125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="15.7265625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" style="9" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" style="9" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" style="9"/>
+    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" t="s">
         <v>79</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" t="s">
         <v>82</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" t="s">
         <v>83</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" t="s">
         <v>89</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" t="s">
         <v>71</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" t="s">
         <v>86</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" t="s">
         <v>76</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" t="s">
         <v>77</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" t="s">
         <v>75</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B15" s="10" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16">
         <v>0.34722222222222221</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" t="s">
         <v>93</v>
       </c>
-      <c r="D17" s="9">
-        <v>0</v>
-      </c>
-      <c r="E17" s="9">
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
         <v>0.27</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18">
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" t="s">
         <v>99</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19">
         <v>298</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" t="s">
         <v>103</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20">
         <v>24450</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20">
         <v>24450</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="9">
-        <v>0</v>
-      </c>
-      <c r="E21" s="9">
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
         <v>55</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
+      <c r="D22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="9">
-        <v>0</v>
-      </c>
-      <c r="E24" s="9">
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="10" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="9">
-        <v>0</v>
-      </c>
-      <c r="E25" s="9">
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="10" t="s">
+      <c r="D26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" t="s">
         <v>17</v>
       </c>
-      <c r="D27" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="10" t="s">
+      <c r="D27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="9">
+      <c r="E28">
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="10" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" t="s">
         <v>23</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="10" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" t="s">
         <v>47</v>
       </c>
-      <c r="D32" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="10" t="s">
+      <c r="D32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B33" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="10" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="10" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" t="s">
         <v>57</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" t="s">
         <v>59</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B39" s="10" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2328,535 +2314,534 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDE04527-9F31-4466-9691-89DE654EA2DE}">
   <dimension ref="A1:F39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.6328125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="15.7265625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" style="9" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" style="9" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" style="9"/>
+    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" t="s">
         <v>79</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" t="s">
         <v>82</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" t="s">
         <v>83</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" t="s">
         <v>89</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" t="s">
         <v>71</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" t="s">
         <v>86</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" t="s">
         <v>76</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" t="s">
         <v>77</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" t="s">
         <v>75</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B15" s="10" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16">
         <v>0.2291667</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" t="s">
         <v>93</v>
       </c>
-      <c r="D17" s="9">
-        <v>0</v>
-      </c>
-      <c r="E17" s="9">
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
         <v>0.23</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18">
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" t="s">
         <v>99</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19">
         <v>298</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" t="s">
         <v>103</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20">
         <v>24450</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20">
         <v>24450</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="9">
-        <v>0</v>
-      </c>
-      <c r="E21" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="9">
-        <v>0</v>
-      </c>
-      <c r="E22" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="9">
-        <v>0</v>
-      </c>
-      <c r="E24" s="9">
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
         <v>103</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="10" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="9">
-        <v>0</v>
-      </c>
-      <c r="E25" s="9">
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="9">
-        <v>0</v>
-      </c>
-      <c r="E26" s="9">
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
         <v>9.1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="10" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" t="s">
         <v>17</v>
       </c>
-      <c r="D27" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="10" t="s">
+      <c r="D27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="10" t="s">
+      <c r="E28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" t="s">
         <v>23</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="10" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" t="s">
         <v>47</v>
       </c>
-      <c r="D32" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="10" t="s">
+      <c r="D32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B33" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="10" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="10" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" t="s">
         <v>57</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" t="s">
         <v>59</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B39" s="10" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2866,535 +2851,534 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21E2476A-44A9-4EA5-A631-010D0DD6FA88}">
   <dimension ref="A1:F39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.6328125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="15.7265625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" style="9" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" style="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" style="9" customWidth="1"/>
-    <col min="11" max="16384" width="8.7265625" style="9"/>
+    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" t="s">
         <v>79</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" t="s">
         <v>82</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" t="s">
         <v>83</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" t="s">
         <v>89</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" t="s">
         <v>71</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" t="s">
         <v>86</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" t="s">
         <v>76</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" t="s">
         <v>77</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" t="s">
         <v>75</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B15" s="10" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16">
         <v>0.2291667</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" t="s">
         <v>93</v>
       </c>
-      <c r="D17" s="9">
-        <v>0</v>
-      </c>
-      <c r="E17" s="9">
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
         <v>2.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18">
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" t="s">
         <v>99</v>
       </c>
-      <c r="D19" s="9">
+      <c r="D19">
         <v>298</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" t="s">
         <v>103</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20">
         <v>24450</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20">
         <v>24450</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="9">
-        <v>0</v>
-      </c>
-      <c r="E21" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="9">
-        <v>0</v>
-      </c>
-      <c r="E22" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="9">
-        <v>0</v>
-      </c>
-      <c r="E24" s="9">
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
         <v>1000</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="10" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="9">
-        <v>0</v>
-      </c>
-      <c r="E25" s="9">
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="9">
-        <v>0</v>
-      </c>
-      <c r="E26" s="9">
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
         <v>9.1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="10" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" t="s">
         <v>17</v>
       </c>
-      <c r="D27" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="10" t="s">
+      <c r="D27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="10" t="s">
+      <c r="E28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" t="s">
         <v>23</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="10" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" t="s">
         <v>47</v>
       </c>
-      <c r="D32" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="10" t="s">
+      <c r="D32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B33" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="10" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="10" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" t="s">
         <v>57</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" t="s">
         <v>59</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B39" s="10" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3402,72 +3386,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="41d9f072-86bf-4c63-b117-debf50ff4701">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3940,23 +3858,96 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="41d9f072-86bf-4c63-b117-debf50ff4701">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74E43103-4BB8-4F2E-AC53-ED5EAA6897C8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+    <ds:schemaRef ds:uri="41d9f072-86bf-4c63-b117-debf50ff4701"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3966,10 +3957,24 @@
     <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
     <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+    <ds:schemaRef ds:uri="41d9f072-86bf-4c63-b117-debf50ff4701"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74E43103-4BB8-4F2E-AC53-ED5EAA6897C8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>